<commit_message>
conducted response time analysis
</commit_message>
<xml_diff>
--- a/src/tools/xil-data-analysis/2023-Hyundai-Ioniq5/output-files/auxiliary-analysis-data.xlsx
+++ b/src/tools/xil-data-analysis/2023-Hyundai-Ioniq5/output-files/auxiliary-analysis-data.xlsx
@@ -5,25 +5,24 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ddas\Documents\deb-anl-xil\src\tools\xil-data-analysis\2023-Hyundai-Ioniq5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ddas\Documents\deb-anl-xil\src\tools\xil-data-analysis\2023-Hyundai-Ioniq5\output-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569356E7-40D4-439E-8411-43BE3CB08BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2002985-131C-414F-BF19-CF59F35A5F1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0-20mph" sheetId="1" r:id="rId1"/>
-    <sheet name="20-40mph" sheetId="2" r:id="rId2"/>
-    <sheet name="30-50mph" sheetId="3" r:id="rId3"/>
-    <sheet name="50-70mph" sheetId="4" r:id="rId4"/>
+    <sheet name="30-50mph" sheetId="3" r:id="rId2"/>
+    <sheet name="50-70mph" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="3">
   <si>
     <t>Accel_Value</t>
   </si>
@@ -38,18 +37,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -65,7 +59,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -88,31 +82,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -418,9 +394,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -434,7 +410,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>0.25</v>
       </c>
@@ -448,7 +424,7 @@
         <v>38.300000000000473</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>-0.25</v>
       </c>
@@ -462,7 +438,7 @@
         <v>39.39999999999776</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>0.5</v>
       </c>
@@ -476,7 +452,7 @@
         <v>19.499999999998892</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>-0.5</v>
       </c>
@@ -490,7 +466,7 @@
         <v>20.899999999998808</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1</v>
       </c>
@@ -504,7 +480,7 @@
         <v>10.299999999999409</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>-1</v>
       </c>
@@ -518,7 +494,7 @@
         <v>12.09999999999974</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1.5</v>
       </c>
@@ -532,7 +508,7 @@
         <v>7.3000000000016598</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>-1.5</v>
       </c>
@@ -546,7 +522,7 @@
         <v>8.9000000000020236</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2</v>
       </c>
@@ -560,7 +536,7 @@
         <v>6.5000000000014779</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>-2</v>
       </c>
@@ -574,7 +550,7 @@
         <v>7.5000000000017053</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2.5</v>
       </c>
@@ -588,7 +564,7 @@
         <v>6.6000000000015007</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>-2.5</v>
       </c>
@@ -602,7 +578,7 @@
         <v>6.4000000000014552</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>3</v>
       </c>
@@ -616,7 +592,7 @@
         <v>6.5000000000014779</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>-3</v>
       </c>
@@ -636,53 +612,53 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>0.25</v>
       </c>
       <c r="B2">
-        <v>0.69999999999996021</v>
+        <v>0.4</v>
       </c>
       <c r="C2">
         <v>0.25</v>
       </c>
       <c r="D2">
-        <v>37.699999999997857</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>35.799999999999997</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>-0.25</v>
       </c>
       <c r="B3">
-        <v>0.39999999999997732</v>
+        <v>0.1999999999999886</v>
       </c>
       <c r="C3">
         <v>-0.25</v>
       </c>
       <c r="D3">
-        <v>40.200000000000003</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>35.1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>0.5</v>
       </c>
@@ -693,80 +669,80 @@
         <v>0.5</v>
       </c>
       <c r="D4">
-        <v>20.100000000000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>19.2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>-0.5</v>
       </c>
       <c r="B5">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="C5">
         <v>-0.5</v>
       </c>
       <c r="D5">
-        <v>22.40000000000401</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>18.499999999998948</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6">
-        <v>0.40000000000009089</v>
+        <v>0.39999999999997732</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6">
-        <v>10.199999999999999</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>9.9000000000013983</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>-1</v>
       </c>
       <c r="B7">
-        <v>0.3</v>
+        <v>0.30000000000006821</v>
       </c>
       <c r="C7">
         <v>-1</v>
       </c>
       <c r="D7">
-        <v>8.6999999999999993</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>9.2000000000020918</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1.5</v>
       </c>
       <c r="B8">
-        <v>0.40000000000009089</v>
+        <v>0.30000000000006821</v>
       </c>
       <c r="C8">
         <v>1.5</v>
       </c>
       <c r="D8">
-        <v>6.8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+        <v>7.1000000000016144</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>-1.5</v>
       </c>
       <c r="B9">
-        <v>0.30000000000006821</v>
+        <v>0.2000000000000455</v>
       </c>
       <c r="C9">
         <v>-1.5</v>
       </c>
       <c r="D9">
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+        <v>6.6000000000015007</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2</v>
       </c>
@@ -777,77 +753,77 @@
         <v>2</v>
       </c>
       <c r="D10">
-        <v>5.8000000000013188</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+        <v>6.100000000001387</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>-2</v>
       </c>
       <c r="B11">
-        <v>0.2000000000000455</v>
+        <v>0.30000000000006821</v>
       </c>
       <c r="C11">
         <v>-2</v>
       </c>
       <c r="D11">
-        <v>5.3000000000012051</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5.6000000000012733</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2.5</v>
       </c>
       <c r="B12">
-        <v>0.40000000000009089</v>
+        <v>0.30000000000006821</v>
       </c>
       <c r="C12">
         <v>2.5</v>
       </c>
       <c r="D12">
-        <v>5.9000000000013424</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5.700000000001296</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>-2.5</v>
       </c>
       <c r="B13">
-        <v>0.30000000000006821</v>
+        <v>0.2000000000000455</v>
       </c>
       <c r="C13">
         <v>-2.5</v>
       </c>
       <c r="D13">
-        <v>4.3000000000009777</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4.7000000000010687</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>3</v>
       </c>
       <c r="B14">
-        <v>0.30000000000006821</v>
+        <v>0.3</v>
       </c>
       <c r="C14">
         <v>3</v>
       </c>
       <c r="D14">
-        <v>5.6000000000012733</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5.5000000000012514</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>-3</v>
       </c>
       <c r="B15">
-        <v>0.2000000000000455</v>
+        <v>0.1</v>
       </c>
       <c r="C15">
         <v>-3</v>
       </c>
       <c r="D15">
-        <v>3.9</v>
+        <v>3.600000000000819</v>
       </c>
     </row>
   </sheetData>
@@ -856,11 +832,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -874,49 +850,49 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>0.25</v>
       </c>
       <c r="B2">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="C2">
         <v>0.25</v>
       </c>
       <c r="D2">
-        <v>35.799999999999997</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>38.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>-0.25</v>
       </c>
       <c r="B3">
-        <v>0.1999999999999886</v>
+        <v>0.2</v>
       </c>
       <c r="C3">
         <v>-0.25</v>
       </c>
       <c r="D3">
-        <v>35.1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>37.299999999999997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>0.5</v>
       </c>
       <c r="B4">
-        <v>0.39999999999997732</v>
+        <v>0.1</v>
       </c>
       <c r="C4">
         <v>0.5</v>
       </c>
       <c r="D4">
-        <v>19.2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>19.399999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>-0.5</v>
       </c>
@@ -927,356 +903,136 @@
         <v>-0.5</v>
       </c>
       <c r="D5">
-        <v>18.499999999998948</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>17.600000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6">
-        <v>0.39999999999997732</v>
+        <v>0.2</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6">
-        <v>9.9000000000013983</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>9.6999999999999993</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>-1</v>
       </c>
       <c r="B7">
-        <v>0.30000000000006821</v>
+        <v>0.2</v>
       </c>
       <c r="C7">
         <v>-1</v>
       </c>
       <c r="D7">
-        <v>9.2000000000020918</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1.5</v>
       </c>
       <c r="B8">
-        <v>0.30000000000006821</v>
+        <v>0.1</v>
       </c>
       <c r="C8">
         <v>1.5</v>
       </c>
       <c r="D8">
-        <v>7.1000000000016144</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>-1.5</v>
       </c>
       <c r="B9">
-        <v>0.2000000000000455</v>
+        <v>0.1</v>
       </c>
       <c r="C9">
         <v>-1.5</v>
       </c>
       <c r="D9">
-        <v>6.6000000000015007</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2</v>
       </c>
       <c r="B10">
-        <v>0.40000000000009089</v>
+        <v>0.1</v>
       </c>
       <c r="C10">
         <v>2</v>
       </c>
       <c r="D10">
-        <v>6.100000000001387</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>-2</v>
       </c>
       <c r="B11">
-        <v>0.30000000000006821</v>
+        <v>0.1</v>
       </c>
       <c r="C11">
         <v>-2</v>
       </c>
       <c r="D11">
-        <v>5.6000000000012733</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2.5</v>
       </c>
       <c r="B12">
-        <v>0.30000000000006821</v>
+        <v>0.1</v>
       </c>
       <c r="C12">
         <v>2.5</v>
       </c>
       <c r="D12">
-        <v>5.700000000001296</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>-2.5</v>
       </c>
       <c r="B13">
-        <v>0.2000000000000455</v>
+        <v>0.1</v>
       </c>
       <c r="C13">
         <v>-2.5</v>
       </c>
       <c r="D13">
-        <v>4.7000000000010687</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>3</v>
       </c>
       <c r="B14">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="C14">
         <v>3</v>
       </c>
       <c r="D14">
-        <v>5.5000000000012514</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>-3</v>
-      </c>
-      <c r="B15">
-        <v>0.1</v>
-      </c>
-      <c r="C15">
-        <v>-3</v>
-      </c>
-      <c r="D15">
-        <v>3.600000000000819</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>0.25</v>
-      </c>
-      <c r="B2">
-        <v>0.2</v>
-      </c>
-      <c r="C2">
-        <v>0.25</v>
-      </c>
-      <c r="D2">
-        <v>38.1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>-0.25</v>
-      </c>
-      <c r="B3">
-        <v>0.2</v>
-      </c>
-      <c r="C3">
-        <v>-0.25</v>
-      </c>
-      <c r="D3">
-        <v>37.299999999999997</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>0.5</v>
-      </c>
-      <c r="B4">
-        <v>0.1</v>
-      </c>
-      <c r="C4">
-        <v>0.5</v>
-      </c>
-      <c r="D4">
-        <v>19.399999999999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>-0.5</v>
-      </c>
-      <c r="B5">
-        <v>0.2</v>
-      </c>
-      <c r="C5">
-        <v>-0.5</v>
-      </c>
-      <c r="D5">
-        <v>17.600000000000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>1</v>
-      </c>
-      <c r="B6">
-        <v>0.2</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6">
-        <v>9.6999999999999993</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>-1</v>
-      </c>
-      <c r="B7">
-        <v>0.2</v>
-      </c>
-      <c r="C7">
-        <v>-1</v>
-      </c>
-      <c r="D7">
-        <v>8.6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>1.5</v>
-      </c>
-      <c r="B8">
-        <v>0.1</v>
-      </c>
-      <c r="C8">
-        <v>1.5</v>
-      </c>
-      <c r="D8">
-        <v>6.9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>-1.5</v>
-      </c>
-      <c r="B9">
-        <v>0.1</v>
-      </c>
-      <c r="C9">
-        <v>-1.5</v>
-      </c>
-      <c r="D9">
-        <v>6.1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>2</v>
-      </c>
-      <c r="B10">
-        <v>0.1</v>
-      </c>
-      <c r="C10">
-        <v>2</v>
-      </c>
-      <c r="D10">
-        <v>5.9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>-2</v>
-      </c>
-      <c r="B11">
-        <v>0.1</v>
-      </c>
-      <c r="C11">
-        <v>-2</v>
-      </c>
-      <c r="D11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>2.5</v>
-      </c>
-      <c r="B12">
-        <v>0.1</v>
-      </c>
-      <c r="C12">
-        <v>2.5</v>
-      </c>
-      <c r="D12">
-        <v>5.9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>-2.5</v>
-      </c>
-      <c r="B13">
-        <v>0.1</v>
-      </c>
-      <c r="C13">
-        <v>-2.5</v>
-      </c>
-      <c r="D13">
-        <v>4.2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>3</v>
-      </c>
-      <c r="B14">
-        <v>0.1</v>
-      </c>
-      <c r="C14">
-        <v>3</v>
-      </c>
-      <c r="D14">
         <v>5.9000000000013424</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>-3</v>
       </c>

</xml_diff>